<commit_message>
chore: add training results and evaluation metrics for ResNet50 scratch 5-seeds experiment
</commit_message>
<xml_diff>
--- a/dataset_cashew.xlsx
+++ b/dataset_cashew.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\KhoaLuanTotNghiep\Resource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4282AE1-2456-4878-A626-DF261D1A0F4A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11822F98-73A2-4A2A-A7E5-3265869AFD67}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11829" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -415,7 +415,15 @@
           <a:p>
             <a:r>
               <a:rPr lang="vi-VN"/>
-              <a:t>Phân bố Data cải tiến (7.464 ảnh)</a:t>
+              <a:t>Phân bố Data cải tiến (7.</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>208</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="vi-VN"/>
+              <a:t> ảnh)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -463,16 +471,16 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1592</c:v>
+                  <c:v>1563</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1415</c:v>
+                  <c:v>1171</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1362</c:v>
+                  <c:v>1312</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1523</c:v>
+                  <c:v>1593</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1572</c:v>
@@ -888,11 +896,11 @@
         <v>6</v>
       </c>
       <c r="G6" s="7">
-        <v>1592</v>
+        <v>1563</v>
       </c>
       <c r="H6" s="8">
         <f>G6/$G$11</f>
-        <v>0.21329046087888531</v>
+        <v>0.21675218416308417</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="12" customHeight="1">
@@ -910,11 +918,11 @@
         <v>7</v>
       </c>
       <c r="G7" s="9">
-        <v>1415</v>
+        <v>1171</v>
       </c>
       <c r="H7" s="10">
         <f>G7/$G$11</f>
-        <v>0.18957663451232584</v>
+        <v>0.16239079184579117</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="12" customHeight="1">
@@ -932,11 +940,11 @@
         <v>8</v>
       </c>
       <c r="G8" s="9">
-        <v>1362</v>
+        <v>1312</v>
       </c>
       <c r="H8" s="10">
         <f>G8/$G$11</f>
-        <v>0.182475884244373</v>
+        <v>0.18194425183747054</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="12" customHeight="1">
@@ -954,11 +962,11 @@
         <v>9</v>
       </c>
       <c r="G9" s="9">
-        <v>1523</v>
+        <v>1593</v>
       </c>
       <c r="H9" s="10">
         <f>G9/$G$11</f>
-        <v>0.20404608788853162</v>
+        <v>0.2209124947996117</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="12" customHeight="1">
@@ -981,7 +989,7 @@
       </c>
       <c r="H10" s="10">
         <f>G10/$G$11</f>
-        <v>0.21061093247588425</v>
+        <v>0.21800027735404243</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="12" customHeight="1">
@@ -990,7 +998,7 @@
       </c>
       <c r="G11" s="13">
         <f>SUM(G6:G10)</f>
-        <v>7464</v>
+        <v>7211</v>
       </c>
       <c r="H11" s="14">
         <f>SUM(H6:H10)</f>

</xml_diff>